<commit_message>
Updated ART 15a and b
ensured that ART start date is not blank before applying to_period
</commit_message>
<xml_diff>
--- a/ART MSF SUMMARY AS AT May 2025.xlsx
+++ b/ART MSF SUMMARY AS AT May 2025.xlsx
@@ -472,7 +472,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Holy Rosary Hospital ART Monthly Summary Form As At May 2025</t>
+          <t>Igboukwu Diocesan Hospital ART Monthly Summary Form As At May 2025</t>
         </is>
       </c>
     </row>
@@ -633,52 +633,52 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="O5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -953,49 +953,49 @@
         <v>0</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="O12" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="P12" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="F12" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="I12" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="J12" s="4" t="n">
-        <v>42</v>
-      </c>
-      <c r="K12" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="L12" s="4" t="n">
-        <v>76</v>
-      </c>
-      <c r="M12" s="4" t="n">
-        <v>66</v>
-      </c>
-      <c r="N12" s="4" t="n">
-        <v>55</v>
-      </c>
-      <c r="O12" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="P12" s="4" t="n">
-        <v>25</v>
-      </c>
       <c r="Q12" s="4" t="n">
-        <v>418</v>
+        <v>255</v>
       </c>
       <c r="R12" s="4" t="n"/>
     </row>
@@ -1009,49 +1009,49 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
         <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F13" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="G13" t="n">
+        <v>25</v>
+      </c>
+      <c r="H13" t="n">
+        <v>54</v>
+      </c>
+      <c r="I13" t="n">
+        <v>60</v>
+      </c>
+      <c r="J13" t="n">
+        <v>59</v>
+      </c>
+      <c r="K13" t="n">
+        <v>70</v>
+      </c>
+      <c r="L13" t="n">
+        <v>46</v>
+      </c>
+      <c r="M13" t="n">
+        <v>32</v>
+      </c>
+      <c r="N13" t="n">
         <v>20</v>
       </c>
-      <c r="H13" t="n">
-        <v>31</v>
-      </c>
-      <c r="I13" t="n">
-        <v>69</v>
-      </c>
-      <c r="J13" t="n">
-        <v>102</v>
-      </c>
-      <c r="K13" t="n">
-        <v>196</v>
-      </c>
-      <c r="L13" t="n">
-        <v>180</v>
-      </c>
-      <c r="M13" t="n">
-        <v>115</v>
-      </c>
-      <c r="N13" t="n">
-        <v>54</v>
-      </c>
       <c r="O13" t="n">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="P13" t="n">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="Q13" t="n">
-        <v>846</v>
+        <v>409</v>
       </c>
     </row>
     <row r="14">
@@ -1106,7 +1106,7 @@
         <v/>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="R14" s="4" t="n"/>
     </row>
@@ -1162,7 +1162,7 @@
         <v/>
       </c>
       <c r="Q15" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16"/>
@@ -1207,16 +1207,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>407</v>
+        <v>250</v>
       </c>
       <c r="D19" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E19" t="n">
-        <v>837</v>
+        <v>402</v>
       </c>
     </row>
     <row r="20">
@@ -1265,16 +1265,16 @@
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>407</v>
+        <v>250</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>837</v>
+        <v>402</v>
       </c>
       <c r="F22" s="4" t="n"/>
     </row>
@@ -1320,16 +1320,16 @@
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>345</v>
+        <v>25</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>741</v>
+        <v>40</v>
       </c>
       <c r="F26" s="4" t="n"/>
     </row>
@@ -1382,13 +1382,13 @@
         <v>0</v>
       </c>
       <c r="C29" t="n">
-        <v>55</v>
+        <v>224</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E29" t="n">
-        <v>89</v>
+        <v>360</v>
       </c>
     </row>
     <row r="30">
@@ -1398,16 +1398,16 @@
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C30" s="4" t="n">
+        <v>249</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E30" s="4" t="n">
         <v>400</v>
-      </c>
-      <c r="D30" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="E30" s="4" t="n">
-        <v>830</v>
       </c>
       <c r="F30" s="4" t="n"/>
     </row>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>1261</v>
+        <v>353</v>
       </c>
       <c r="C34" s="4" t="n"/>
     </row>
@@ -1449,7 +1449,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>3</v>
+        <v>311</v>
       </c>
     </row>
     <row r="36"/>
@@ -1554,52 +1554,52 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="C39" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="E39" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="I39" t="n">
-        <v/>
+        <v>2</v>
       </c>
       <c r="J39" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="L39" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="M39" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="N39" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="O39" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="P39" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q39" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="40">
@@ -1633,7 +1633,7 @@
         <v>0</v>
       </c>
       <c r="J40" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K40" s="4" t="n">
         <v>1</v>
@@ -1645,7 +1645,7 @@
         <v>0</v>
       </c>
       <c r="N40" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O40" s="4" t="n">
         <v>0</v>
@@ -1654,7 +1654,7 @@
         <v>0</v>
       </c>
       <c r="Q40" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R40" s="4" t="n"/>
     </row>
@@ -1821,7 +1821,7 @@
         <v/>
       </c>
       <c r="Q43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44">
@@ -1876,7 +1876,7 @@
         <v/>
       </c>
       <c r="Q44" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R44" s="4" t="n"/>
     </row>
@@ -1985,49 +1985,49 @@
         <v>0</v>
       </c>
       <c r="C48" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G48" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H48" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="I48" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="J48" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="K48" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="L48" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="M48" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="N48" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="O48" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="H48" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="I48" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="J48" s="4" t="n">
-        <v>34</v>
-      </c>
-      <c r="K48" s="4" t="n">
-        <v>39</v>
-      </c>
-      <c r="L48" s="4" t="n">
-        <v>64</v>
-      </c>
-      <c r="M48" s="4" t="n">
-        <v>56</v>
-      </c>
-      <c r="N48" s="4" t="n">
-        <v>47</v>
-      </c>
-      <c r="O48" s="4" t="n">
-        <v>25</v>
-      </c>
       <c r="P48" s="4" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="Q48" s="4" t="n">
-        <v>348</v>
+        <v>230</v>
       </c>
       <c r="R48" s="4" t="n"/>
     </row>
@@ -2041,49 +2041,49 @@
         <v>0</v>
       </c>
       <c r="C49" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D49" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E49" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F49" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="G49" t="n">
+        <v>24</v>
+      </c>
+      <c r="H49" t="n">
+        <v>51</v>
+      </c>
+      <c r="I49" t="n">
+        <v>53</v>
+      </c>
+      <c r="J49" t="n">
+        <v>50</v>
+      </c>
+      <c r="K49" t="n">
+        <v>63</v>
+      </c>
+      <c r="L49" t="n">
+        <v>43</v>
+      </c>
+      <c r="M49" t="n">
+        <v>27</v>
+      </c>
+      <c r="N49" t="n">
+        <v>18</v>
+      </c>
+      <c r="O49" t="n">
+        <v>14</v>
+      </c>
+      <c r="P49" t="n">
         <v>13</v>
       </c>
-      <c r="H49" t="n">
-        <v>25</v>
-      </c>
-      <c r="I49" t="n">
-        <v>60</v>
-      </c>
-      <c r="J49" t="n">
-        <v>87</v>
-      </c>
-      <c r="K49" t="n">
-        <v>165</v>
-      </c>
-      <c r="L49" t="n">
-        <v>152</v>
-      </c>
-      <c r="M49" t="n">
-        <v>96</v>
-      </c>
-      <c r="N49" t="n">
-        <v>48</v>
-      </c>
-      <c r="O49" t="n">
-        <v>27</v>
-      </c>
-      <c r="P49" t="n">
-        <v>22</v>
-      </c>
       <c r="Q49" t="n">
-        <v>712</v>
+        <v>365</v>
       </c>
     </row>
     <row r="50">
@@ -2138,7 +2138,7 @@
         <v/>
       </c>
       <c r="Q50" s="4" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="R50" s="4" t="n"/>
     </row>
@@ -2194,7 +2194,7 @@
         <v/>
       </c>
       <c r="Q51" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52"/>
@@ -2326,7 +2326,7 @@
         <v>0</v>
       </c>
       <c r="K55" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L55" t="n">
         <v>0</v>
@@ -2335,7 +2335,7 @@
         <v>0</v>
       </c>
       <c r="N55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O55" t="n">
         <v>0</v>
@@ -2344,7 +2344,7 @@
         <v>0</v>
       </c>
       <c r="Q55" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -2372,10 +2372,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I56" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J56" s="4" t="n">
         <v>0</v>
@@ -2387,19 +2387,19 @@
         <v>0</v>
       </c>
       <c r="M56" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N56" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O56" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P56" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q56" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="R56" s="4" t="n"/>
     </row>
@@ -2730,49 +2730,49 @@
         <v>0</v>
       </c>
       <c r="C64" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D64" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E64" s="4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="H64" s="4" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="I64" s="4" t="n">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="J64" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="K64" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="L64" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="K64" s="4" t="n">
-        <v>37</v>
-      </c>
-      <c r="L64" s="4" t="n">
-        <v>58</v>
-      </c>
       <c r="M64" s="4" t="n">
-        <v>53</v>
+        <v>12</v>
       </c>
       <c r="N64" s="4" t="n">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="O64" s="4" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="P64" s="4" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="Q64" s="4" t="n">
-        <v>321</v>
+        <v>209</v>
       </c>
       <c r="R64" s="4" t="n"/>
     </row>
@@ -2786,49 +2786,49 @@
         <v>0</v>
       </c>
       <c r="C65" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D65" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E65" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F65" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G65" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="H65" t="n">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="I65" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="J65" t="n">
-        <v>80</v>
+        <v>47</v>
       </c>
       <c r="K65" t="n">
-        <v>158</v>
+        <v>57</v>
       </c>
       <c r="L65" t="n">
-        <v>144</v>
+        <v>38</v>
       </c>
       <c r="M65" t="n">
-        <v>94</v>
+        <v>25</v>
       </c>
       <c r="N65" t="n">
-        <v>47</v>
+        <v>18</v>
       </c>
       <c r="O65" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="P65" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="Q65" t="n">
-        <v>676</v>
+        <v>338</v>
       </c>
     </row>
     <row r="66">
@@ -2883,7 +2883,7 @@
         <v/>
       </c>
       <c r="Q66" s="4" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="R66" s="4" t="n"/>
     </row>
@@ -2939,7 +2939,7 @@
         <v/>
       </c>
       <c r="Q67" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68"/>
@@ -3071,7 +3071,7 @@
         <v>0</v>
       </c>
       <c r="K71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L71" t="n">
         <v>0</v>
@@ -3080,7 +3080,7 @@
         <v>0</v>
       </c>
       <c r="N71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O71" t="n">
         <v>0</v>
@@ -3089,7 +3089,7 @@
         <v>0</v>
       </c>
       <c r="Q71" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -3138,13 +3138,13 @@
         <v>0</v>
       </c>
       <c r="O72" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P72" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q72" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R72" s="4" t="n"/>
     </row>
@@ -3487,7 +3487,7 @@
         <v>0</v>
       </c>
       <c r="G80" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H80" s="4" t="n">
         <v>0</v>
@@ -3496,13 +3496,13 @@
         <v>0</v>
       </c>
       <c r="J80" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K80" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L80" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M80" s="4" t="n">
         <v>0</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="Q80" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="R80" s="4" t="n"/>
     </row>
@@ -3534,10 +3534,10 @@
         <v>0</v>
       </c>
       <c r="D81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F81" t="n">
         <v>0</v>
@@ -3546,16 +3546,16 @@
         <v>0</v>
       </c>
       <c r="H81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I81" t="n">
         <v>0</v>
       </c>
       <c r="J81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L81" t="n">
         <v>0</v>
@@ -3564,7 +3564,7 @@
         <v>0</v>
       </c>
       <c r="N81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O81" t="n">
         <v>0</v>
@@ -3573,7 +3573,7 @@
         <v>0</v>
       </c>
       <c r="Q81" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="82"/>
@@ -3699,7 +3699,7 @@
         <v>0</v>
       </c>
       <c r="I85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J85" t="n">
         <v>0</v>
@@ -3723,7 +3723,7 @@
         <v>0</v>
       </c>
       <c r="Q85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -3760,7 +3760,7 @@
         <v>0</v>
       </c>
       <c r="K86" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L86" s="4" t="n">
         <v>0</v>
@@ -3778,7 +3778,7 @@
         <v>0</v>
       </c>
       <c r="Q86" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R86" s="4" t="n"/>
     </row>
@@ -3976,7 +3976,7 @@
         <v>0</v>
       </c>
       <c r="N91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O91" t="n">
         <v>0</v>
@@ -3985,7 +3985,7 @@
         <v>0</v>
       </c>
       <c r="Q91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92"/>
@@ -4099,43 +4099,43 @@
         <v>0</v>
       </c>
       <c r="E95" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F95" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G95" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H95" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I95" t="n">
         <v>5</v>
       </c>
       <c r="J95" t="n">
+        <v>8</v>
+      </c>
+      <c r="K95" t="n">
         <v>10</v>
       </c>
-      <c r="K95" t="n">
-        <v>9</v>
-      </c>
       <c r="L95" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="M95" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="N95" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="O95" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P95" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="Q95" t="n">
-        <v>88</v>
+        <v>57</v>
       </c>
     </row>
     <row r="96">
@@ -4148,7 +4148,7 @@
         <v>0</v>
       </c>
       <c r="C96" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D96" s="4" t="n">
         <v>0</v>
@@ -4157,40 +4157,40 @@
         <v>0</v>
       </c>
       <c r="F96" s="4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G96" s="4" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H96" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I96" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="J96" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="K96" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="L96" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="M96" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N96" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O96" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P96" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="I96" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="J96" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="K96" s="4" t="n">
-        <v>42</v>
-      </c>
-      <c r="L96" s="4" t="n">
-        <v>38</v>
-      </c>
-      <c r="M96" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="N96" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="O96" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="P96" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="Q96" s="4" t="n">
-        <v>187</v>
+        <v>85</v>
       </c>
       <c r="R96" s="4" t="n"/>
     </row>
@@ -4299,7 +4299,7 @@
         <v>0</v>
       </c>
       <c r="C100" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D100" s="4" t="n">
         <v>0</v>
@@ -4314,13 +4314,13 @@
         <v>1</v>
       </c>
       <c r="H100" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I100" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J100" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K100" s="4" t="n">
         <v>2</v>
@@ -4329,19 +4329,19 @@
         <v>1</v>
       </c>
       <c r="M100" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N100" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O100" s="4" t="n">
         <v>0</v>
       </c>
       <c r="P100" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q100" s="4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="R100" s="4" t="n"/>
     </row>
@@ -4355,49 +4355,49 @@
         <v>0</v>
       </c>
       <c r="C101" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F101" t="n">
         <v>1</v>
       </c>
       <c r="G101" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I101" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J101" t="n">
+        <v>5</v>
+      </c>
+      <c r="K101" t="n">
+        <v>0</v>
+      </c>
+      <c r="L101" t="n">
+        <v>4</v>
+      </c>
+      <c r="M101" t="n">
+        <v>0</v>
+      </c>
+      <c r="N101" t="n">
+        <v>1</v>
+      </c>
+      <c r="O101" t="n">
+        <v>0</v>
+      </c>
+      <c r="P101" t="n">
         <v>2</v>
       </c>
-      <c r="K101" t="n">
-        <v>1</v>
-      </c>
-      <c r="L101" t="n">
-        <v>0</v>
-      </c>
-      <c r="M101" t="n">
-        <v>1</v>
-      </c>
-      <c r="N101" t="n">
-        <v>1</v>
-      </c>
-      <c r="O101" t="n">
-        <v>0</v>
-      </c>
-      <c r="P101" t="n">
-        <v>0</v>
-      </c>
       <c r="Q101" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="102"/>
@@ -4511,43 +4511,43 @@
         <v>1</v>
       </c>
       <c r="E105" t="n">
+        <v>1</v>
+      </c>
+      <c r="F105" t="n">
+        <v>1</v>
+      </c>
+      <c r="G105" t="n">
         <v>9</v>
       </c>
-      <c r="F105" t="n">
+      <c r="H105" t="n">
+        <v>22</v>
+      </c>
+      <c r="I105" t="n">
+        <v>30</v>
+      </c>
+      <c r="J105" t="n">
+        <v>34</v>
+      </c>
+      <c r="K105" t="n">
+        <v>28</v>
+      </c>
+      <c r="L105" t="n">
+        <v>18</v>
+      </c>
+      <c r="M105" t="n">
         <v>9</v>
       </c>
-      <c r="G105" t="n">
-        <v>13</v>
-      </c>
-      <c r="H105" t="n">
-        <v>12</v>
-      </c>
-      <c r="I105" t="n">
-        <v>20</v>
-      </c>
-      <c r="J105" t="n">
-        <v>38</v>
-      </c>
-      <c r="K105" t="n">
-        <v>47</v>
-      </c>
-      <c r="L105" t="n">
-        <v>72</v>
-      </c>
-      <c r="M105" t="n">
-        <v>62</v>
-      </c>
       <c r="N105" t="n">
-        <v>51</v>
+        <v>11</v>
       </c>
       <c r="O105" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="P105" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="Q105" t="n">
-        <v>386</v>
+        <v>171</v>
       </c>
     </row>
     <row r="106">
@@ -4560,49 +4560,49 @@
         <v>0</v>
       </c>
       <c r="C106" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D106" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E106" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F106" s="4" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="G106" s="4" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="H106" s="4" t="n">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="I106" s="4" t="n">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="J106" s="4" t="n">
-        <v>93</v>
+        <v>30</v>
       </c>
       <c r="K106" s="4" t="n">
-        <v>191</v>
+        <v>36</v>
       </c>
       <c r="L106" s="4" t="n">
-        <v>176</v>
+        <v>23</v>
       </c>
       <c r="M106" s="4" t="n">
-        <v>108</v>
+        <v>15</v>
       </c>
       <c r="N106" s="4" t="n">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="O106" s="4" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="P106" s="4" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="Q106" s="4" t="n">
-        <v>794</v>
+        <v>234</v>
       </c>
       <c r="R106" s="4" t="n"/>
     </row>
@@ -4726,19 +4726,19 @@
         <v>0</v>
       </c>
       <c r="H110" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I110" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J110" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K110" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L110" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M110" s="4" t="n">
         <v>0</v>
@@ -4750,10 +4750,10 @@
         <v>0</v>
       </c>
       <c r="P110" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q110" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R110" s="4" t="n"/>
     </row>
@@ -4779,22 +4779,22 @@
         <v>0</v>
       </c>
       <c r="G111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H111" t="n">
         <v>0</v>
       </c>
       <c r="I111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J111" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K111" t="n">
         <v>0</v>
       </c>
       <c r="L111" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M111" t="n">
         <v>0</v>
@@ -4806,10 +4806,10 @@
         <v>0</v>
       </c>
       <c r="P111" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q111" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="112"/>
@@ -4920,46 +4920,46 @@
         <v>0</v>
       </c>
       <c r="D115" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E115" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F115" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G115" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="H115" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I115" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="J115" t="n">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="K115" t="n">
-        <v>46</v>
+        <v>1</v>
       </c>
       <c r="L115" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="M115" t="n">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="N115" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="O115" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="P115" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="Q115" t="n">
-        <v>366</v>
+        <v>5</v>
       </c>
     </row>
     <row r="116">
@@ -4972,49 +4972,49 @@
         <v>0</v>
       </c>
       <c r="C116" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D116" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E116" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F116" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G116" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H116" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I116" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J116" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K116" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="D116" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E116" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F116" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="G116" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="H116" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="I116" s="4" t="n">
-        <v>58</v>
-      </c>
-      <c r="J116" s="4" t="n">
-        <v>92</v>
-      </c>
-      <c r="K116" s="4" t="n">
-        <v>187</v>
-      </c>
       <c r="L116" s="4" t="n">
-        <v>173</v>
+        <v>1</v>
       </c>
       <c r="M116" s="4" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="N116" s="4" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="O116" s="4" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="P116" s="4" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="Q116" s="4" t="n">
-        <v>778</v>
+        <v>8</v>
       </c>
       <c r="R116" s="4" t="n"/>
     </row>

</xml_diff>